<commit_message>
feat: Implement optimized SDV imputation strategy and hybrid imputation system
- Added `optimize_sdv_imputation.py` for enhanced imputation using SDV's capabilities.
- Created `run_pipeline.py` to preprocess diabetes datasets into a machine learning-ready format.
- Developed `sdv_imputation_test.py` to compare various SDV imputation methods and evaluate their performance.
- Introduced `smart_hybrid_imputation.py` for a smart hybrid imputation system that selects the best method based on data characteristics.
- Enhanced documentation and comments throughout the code for better understanding and usability.
</commit_message>
<xml_diff>
--- a/Reference_NMB.xlsx
+++ b/Reference_NMB.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maadh\OneDrive\Desktop\PhobosQ\poornima-ML\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/065714efc4fd34e9/Desktop/PhobosQ/poornima-ML/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12644025-090D-4309-8154-D7B54208DAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="1" xr2:uid="{5CAC90CE-3BD8-4DB6-BA32-A6D0BF4ECD9E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{5CAC90CE-3BD8-4DB6-BA32-A6D0BF4ECD9E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>